<commit_message>
added glacierra_secondary tileset in porytiles format
</commit_message>
<xml_diff>
--- a/data/tilesets/decompiled/Porytiles Template.xlsx
+++ b/data/tilesets/decompiled/Porytiles Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\heracross1991\current-projects\pokemon-seel-version\data\tilesets\decompiled\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{8647A00A-FD1E-4247-845A-4BB19EBAD747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A9DDC7-F096-47DE-9310-4A0B0DB7C0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{5AC83084-0AAA-4FBC-A423-071F15440E35}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{5AC83084-0AAA-4FBC-A423-071F15440E35}"/>
   </bookViews>
   <sheets>
     <sheet name="Porytiles Commands" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="48">
   <si>
     <t>general_seel_version</t>
   </si>
@@ -158,10 +158,31 @@
     <t xml:space="preserve">Compile Secondary </t>
   </si>
   <si>
-    <t>test</t>
-  </si>
-  <si>
     <t>~/current-projects/pokemon-seel-version/data/tilesets/decompiled/</t>
+  </si>
+  <si>
+    <t>pyroden</t>
+  </si>
+  <si>
+    <t>dunemire_desert_general</t>
+  </si>
+  <si>
+    <t>dunemire_desert_secondary</t>
+  </si>
+  <si>
+    <t>murkwell_bog</t>
+  </si>
+  <si>
+    <t>verdant_hallow</t>
+  </si>
+  <si>
+    <t>voltbrook_town</t>
+  </si>
+  <si>
+    <t>route_6</t>
+  </si>
+  <si>
+    <t>glacierra_secondary</t>
   </si>
 </sst>
 </file>
@@ -223,7 +244,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -420,19 +441,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -447,7 +455,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -480,11 +488,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -911,7 +918,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5672F8DD-25AC-4492-B1F4-AA4469879AE4}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -932,6 +939,16 @@
         <v>17</v>
       </c>
     </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -939,10 +956,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCBEBE4F-3BE5-4CA4-911B-1F9615EB5F0B}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -958,6 +975,41 @@
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -983,21 +1035,21 @@
   <sheetData>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="30"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
       <c r="E3" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26" t="s">
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1006,7 +1058,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>19</v>
@@ -1014,13 +1066,13 @@
       <c r="E4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26" t="s">
+      <c r="G4" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1028,11 +1080,11 @@
       <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="24" t="str">
+      <c r="B5" s="23" t="str">
         <f>B4</f>
-        <v>stratoscape_primary</v>
-      </c>
-      <c r="C5" s="25" t="s">
+        <v>general_seel_version</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1042,7 +1094,7 @@
       </c>
       <c r="B6" s="13" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B1," ",G3,"data/tilesets/primary/",B4," ",G4,B5," ",G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles compile-primary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/primary/stratoscape_primary ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/stratoscape_primary ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles compile-primary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/primary/general_seel_version ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/general_seel_version ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>18</v>
@@ -1050,18 +1102,18 @@
     </row>
     <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="30"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="29"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="18" t="s">
-        <v>39</v>
+      <c r="B9" t="s">
+        <v>47</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>19</v>
@@ -1071,11 +1123,11 @@
       <c r="A10" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="22" t="str">
+      <c r="B10" s="21" t="str">
         <f>B9</f>
-        <v>test</v>
-      </c>
-      <c r="C10" s="23" t="s">
+        <v>glacierra_secondary</v>
+      </c>
+      <c r="C10" s="22" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1083,7 +1135,7 @@
       <c r="A11" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C11" s="6" t="s">
@@ -1096,7 +1148,7 @@
       </c>
       <c r="B12" s="15" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B2," ",G3,"data/tilesets/secondary/",B9," ",G4,B10," ",G4,B11," ",G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles compile-secondary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/secondary/test ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/test ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/general_seel_version ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles compile-secondary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/secondary/glacierra_secondary ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/glacierra_secondary ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/general_seel_version ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>18</v>
@@ -1104,18 +1156,18 @@
     </row>
     <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="29"/>
-      <c r="C14" s="30"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="29"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>20</v>
@@ -1125,11 +1177,11 @@
       <c r="A16" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="24" t="str">
+      <c r="B16" s="23" t="str">
         <f>B15</f>
-        <v>stratoscape_primary</v>
-      </c>
-      <c r="C16" s="25" t="s">
+        <v>general_seel_version</v>
+      </c>
+      <c r="C16" s="24" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1139,7 +1191,7 @@
       </c>
       <c r="B17" s="13" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B3," ",G4,'Inputs-Outputs'!B15," ",'Inputs-Outputs'!G3,"data/tilesets/primary/",B16," ",G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles decompile-primary -o ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/stratoscape_primary ~/current-projects/pokemon-seel-version/data/tilesets/primary/stratoscape_primary ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles decompile-primary -o ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/general_seel_version ~/current-projects/pokemon-seel-version/data/tilesets/primary/general_seel_version ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>18</v>
@@ -1147,18 +1199,18 @@
     </row>
     <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="29"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="18" t="s">
-        <v>13</v>
+      <c r="B20" t="s">
+        <v>47</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>20</v>
@@ -1168,11 +1220,11 @@
       <c r="A21" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="22" t="str">
+      <c r="B21" s="21" t="str">
         <f>B20</f>
-        <v>dominion_city</v>
-      </c>
-      <c r="C21" s="23" t="s">
+        <v>glacierra_secondary</v>
+      </c>
+      <c r="C21" s="22" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1180,7 +1232,7 @@
       <c r="A22" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C22" s="6" t="s">
@@ -1193,7 +1245,7 @@
       </c>
       <c r="B23" s="15" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B4,," ",'Inputs-Outputs'!G4,'Inputs-Outputs'!B20," ",'Inputs-Outputs'!G3,"data/tilesets/secondary/",'Inputs-Outputs'!B21," ",'Inputs-Outputs'!G3,"data/tilesets/primary/",'Inputs-Outputs'!B22," ",'Inputs-Outputs'!G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles decompile-secondary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/dominion_city ~/current-projects/pokemon-seel-version/data/tilesets/secondary/dominion_city ~/current-projects/pokemon-seel-version/data/tilesets/primary/general_seel_version ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles decompile-secondary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/glacierra_secondary ~/current-projects/pokemon-seel-version/data/tilesets/secondary/glacierra_secondary ~/current-projects/pokemon-seel-version/data/tilesets/primary/general_seel_version ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>18</v>
@@ -1201,10 +1253,10 @@
     </row>
     <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="20" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
map changes. Adding routes to stratoscape
</commit_message>
<xml_diff>
--- a/data/tilesets/decompiled/Porytiles Template.xlsx
+++ b/data/tilesets/decompiled/Porytiles Template.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\heracross1991\current-projects\pokemon-seel-version\data\tilesets\decompiled\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB35887-9B64-4D65-A284-CF2CD4F51063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56379EFA-8304-4335-8569-718CA807B17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{5AC83084-0AAA-4FBC-A423-071F15440E35}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{5AC83084-0AAA-4FBC-A423-071F15440E35}"/>
   </bookViews>
   <sheets>
     <sheet name="Porytiles Commands" sheetId="1" r:id="rId1"/>
     <sheet name="Primary Tilesets" sheetId="3" r:id="rId2"/>
     <sheet name="Secondary Tilesets" sheetId="4" r:id="rId3"/>
-    <sheet name="Inputs-Outputs" sheetId="2" r:id="rId4"/>
+    <sheet name="Projects" sheetId="5" r:id="rId4"/>
+    <sheet name="Inputs-Outputs" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="52">
   <si>
     <t>general_seel_version</t>
   </si>
@@ -158,9 +159,6 @@
     <t xml:space="preserve">Compile Secondary </t>
   </si>
   <si>
-    <t>~/current-projects/pokemon-seel-version/data/tilesets/decompiled/</t>
-  </si>
-  <si>
     <t>pyroden</t>
   </si>
   <si>
@@ -185,7 +183,19 @@
     <t>glacierra_secondary</t>
   </si>
   <si>
-    <t>stratoscape_secondary</t>
+    <t>~/old-projects/pokeemerald_froversion/</t>
+  </si>
+  <si>
+    <t>mount_pyroden</t>
+  </si>
+  <si>
+    <t>~/old-projects/pokeemerald_froversion/data/tilesets/decompiled/</t>
+  </si>
+  <si>
+    <t>summitgeneral</t>
+  </si>
+  <si>
+    <t>summitcity</t>
   </si>
 </sst>
 </file>
@@ -458,7 +468,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -519,6 +529,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -921,7 +932,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5672F8DD-25AC-4492-B1F4-AA4469879AE4}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -944,12 +955,17 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -982,37 +998,37 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1021,6 +1037,26 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A82A7AC-7202-4BA8-9B8F-6376872FEE55}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D27F6184-4E3A-4B6F-BEAB-EFDFF6B4C96D}">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
@@ -1047,7 +1083,7 @@
         <v>25</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="H3" s="25"/>
       <c r="I3" s="25"/>
@@ -1061,7 +1097,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>19</v>
@@ -1070,7 +1106,7 @@
         <v>26</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="H4" s="25"/>
       <c r="I4" s="25"/>
@@ -1085,7 +1121,7 @@
       </c>
       <c r="B5" s="23" t="str">
         <f>B4</f>
-        <v>stratoscape_primary</v>
+        <v>summitgeneral</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>24</v>
@@ -1097,7 +1133,7 @@
       </c>
       <c r="B6" s="13" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B1," ",G3,"data/tilesets/primary/",B4," ",G4,B5," ",G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles compile-primary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/primary/stratoscape_primary ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/stratoscape_primary ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles compile-primary -Wall -o ~/old-projects/pokeemerald_froversion/data/tilesets/primary/summitgeneral ~/old-projects/pokeemerald_froversion/data/tilesets/decompiled/summitgeneral ~/old-projects/pokeemerald_froversion/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>18</v>
@@ -1115,8 +1151,8 @@
       <c r="A9" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B9" t="s">
-        <v>48</v>
+      <c r="B9" s="30" t="s">
+        <v>51</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>19</v>
@@ -1128,7 +1164,7 @@
       </c>
       <c r="B10" s="21" t="str">
         <f>B9</f>
-        <v>stratoscape_secondary</v>
+        <v>summitcity</v>
       </c>
       <c r="C10" s="22" t="s">
         <v>24</v>
@@ -1139,7 +1175,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>21</v>
@@ -1151,7 +1187,7 @@
       </c>
       <c r="B12" s="15" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B2," ",G3,"data/tilesets/secondary/",B9," ",G4,B10," ",G4,B11," ",G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles compile-secondary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/secondary/stratoscape_secondary ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/stratoscape_secondary ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/stratoscape_primary ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles compile-secondary -Wall -o ~/old-projects/pokeemerald_froversion/data/tilesets/secondary/summitcity ~/old-projects/pokeemerald_froversion/data/tilesets/decompiled/summitcity ~/old-projects/pokeemerald_froversion/data/tilesets/decompiled/summitgeneral ~/old-projects/pokeemerald_froversion/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>18</v>
@@ -1170,7 +1206,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>20</v>
@@ -1182,19 +1218,19 @@
       </c>
       <c r="B16" s="23" t="str">
         <f>B15</f>
-        <v>stratoscape_primary</v>
+        <v>summitgeneral</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B17" s="13" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B3," ",G4,'Inputs-Outputs'!B15," ",'Inputs-Outputs'!G3,"data/tilesets/primary/",B16," ",G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles decompile-primary -o ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/stratoscape_primary ~/current-projects/pokemon-seel-version/data/tilesets/primary/stratoscape_primary ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles decompile-primary -o ~/old-projects/pokeemerald_froversion/data/tilesets/decompiled/summitgeneral ~/old-projects/pokeemerald_froversion/data/tilesets/primary/summitgeneral ~/old-projects/pokeemerald_froversion/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>18</v>
@@ -1212,8 +1248,8 @@
       <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B20" t="s">
-        <v>48</v>
+      <c r="B20" s="30" t="s">
+        <v>51</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>20</v>
@@ -1225,7 +1261,7 @@
       </c>
       <c r="B21" s="21" t="str">
         <f>B20</f>
-        <v>stratoscape_secondary</v>
+        <v>summitcity</v>
       </c>
       <c r="C21" s="22" t="s">
         <v>24</v>
@@ -1236,7 +1272,7 @@
         <v>12</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>21</v>
@@ -1248,7 +1284,7 @@
       </c>
       <c r="B23" s="15" t="str">
         <f>_xlfn.CONCAT('Porytiles Commands'!B4,," ",'Inputs-Outputs'!G4,'Inputs-Outputs'!B20," ",'Inputs-Outputs'!G3,"data/tilesets/secondary/",'Inputs-Outputs'!B21," ",'Inputs-Outputs'!G3,"data/tilesets/primary/",'Inputs-Outputs'!B22," ",'Inputs-Outputs'!G3,"include/constants/metatile_behaviors.h")</f>
-        <v>porytiles decompile-secondary -Wall -o ~/current-projects/pokemon-seel-version/data/tilesets/decompiled/stratoscape_secondary ~/current-projects/pokemon-seel-version/data/tilesets/secondary/stratoscape_secondary ~/current-projects/pokemon-seel-version/data/tilesets/primary/stratoscape_primary ~/current-projects/pokemon-seel-version/include/constants/metatile_behaviors.h</v>
+        <v>porytiles decompile-secondary -Wall -o ~/old-projects/pokeemerald_froversion/data/tilesets/decompiled/summitcity ~/old-projects/pokeemerald_froversion/data/tilesets/secondary/summitcity ~/old-projects/pokeemerald_froversion/data/tilesets/primary/summitgeneral ~/old-projects/pokeemerald_froversion/include/constants/metatile_behaviors.h</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Added power plant tileset
</commit_message>
<xml_diff>
--- a/data/tilesets/decompiled/Porytiles Template.xlsx
+++ b/data/tilesets/decompiled/Porytiles Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\heracross1991\current-projects\pokemon-seel-version\data\tilesets\decompiled\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\decomp\pokemon-seel-version\data\tilesets\decompiled\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB35887-9B64-4D65-A284-CF2CD4F51063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1C11B2-6603-46A5-9C8E-C97E47636DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{5AC83084-0AAA-4FBC-A423-071F15440E35}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="3" xr2:uid="{5AC83084-0AAA-4FBC-A423-071F15440E35}"/>
   </bookViews>
   <sheets>
     <sheet name="Porytiles Commands" sheetId="1" r:id="rId1"/>
@@ -854,14 +854,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2225F7C9-C23D-43CA-BA65-488100D8E53D}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -872,7 +872,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
@@ -883,7 +883,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>36</v>
       </c>
@@ -894,7 +894,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
@@ -905,13 +905,13 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
     </row>
   </sheetData>
@@ -922,32 +922,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5672F8DD-25AC-4492-B1F4-AA4469879AE4}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -960,57 +960,57 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCBEBE4F-3BE5-4CA4-911B-1F9615EB5F0B}">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -1026,18 +1026,18 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A2:K25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.28515625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="67.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="10"/>
-    <col min="5" max="5" width="26.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="10"/>
+    <col min="1" max="1" width="30.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.33203125" style="11" customWidth="1"/>
+    <col min="3" max="3" width="67.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="10"/>
+    <col min="5" max="5" width="26.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="10"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="27" t="s">
         <v>1</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="124.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="124.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
@@ -1103,15 +1103,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="27" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="28"/>
       <c r="C8" s="29"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>2</v>
       </c>
@@ -1122,7 +1122,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>3</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>8</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
         <v>4</v>
       </c>
@@ -1157,15 +1157,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="27" t="s">
         <v>6</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="29"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>9</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>10</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="12" t="s">
         <v>4</v>
       </c>
@@ -1200,15 +1200,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="27" t="s">
         <v>7</v>
       </c>
       <c r="B19" s="28"/>
       <c r="C19" s="29"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
         <v>11</v>
       </c>
@@ -1231,7 +1231,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>12</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="135.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="12" t="s">
         <v>4</v>
       </c>
@@ -1254,8 +1254,8 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>23</v>
       </c>

</xml_diff>